<commit_message>
Initial commit - Selenium Cucumber framework
</commit_message>
<xml_diff>
--- a/src/test/resources/ApplicationTableData.xlsx
+++ b/src/test/resources/ApplicationTableData.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1848" uniqueCount="83">
   <si>
     <t>ApplicationNo</t>
   </si>
@@ -259,6 +259,54 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>APP1225-100000207</t>
+  </si>
+  <si>
+    <t>Bhargavi Mantha
+8906763229</t>
+  </si>
+  <si>
+    <t>Pharmacy Trainee</t>
+  </si>
+  <si>
+    <t>22 Dec 2025</t>
+  </si>
+  <si>
+    <t>APP1225-100000216</t>
+  </si>
+  <si>
+    <t>Albert
+8745129696</t>
+  </si>
+  <si>
+    <t>Arya A (arya)
+Source</t>
+  </si>
+  <si>
+    <t>23 Dec 2025</t>
+  </si>
+  <si>
+    <t>APP1225-100000215</t>
+  </si>
+  <si>
+    <t>Roger
+9458946584</t>
+  </si>
+  <si>
+    <t>APP1225-100000214</t>
+  </si>
+  <si>
+    <t>Roberts
+7988965198</t>
+  </si>
+  <si>
+    <t>APP1225-100000209</t>
+  </si>
+  <si>
+    <t>Kaseem Ram
+9885348778</t>
   </si>
 </sst>
 </file>
@@ -614,13 +662,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>39</v>
@@ -629,21 +677,21 @@
         <v>39</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>67</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>39</v>
@@ -652,41 +700,41 @@
         <v>39</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>13</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>39</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>13</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>9</v>
@@ -701,145 +749,145 @@
         <v>44</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>28</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>68</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>68</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>68</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>68</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>